<commit_message>
site build 2026-10-08 21:40
</commit_message>
<xml_diff>
--- a/models/sovereigns/Ukraine_Sovereign_Model.xlsx
+++ b/models/sovereigns/Ukraine_Sovereign_Model.xlsx
@@ -652,7 +652,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>National Bank of Ukraine</t>
+          <t>NBU key rate decision (+50 bps)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -700,12 +700,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>State Statistics Service of Ukraine (Ukrstat)</t>
+          <t>Ukrstat</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>10-Sep-26</t>
+          <t>Sep-26</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -739,11 +739,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -778,7 +774,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>end-2025</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -793,7 +789,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>State and state-guaranteed debt</t>
+          <t>state debt</t>
         </is>
       </c>
     </row>
@@ -843,11 +839,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -929,11 +921,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -991,7 +979,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>National Bank of Ukraine</t>
+          <t>NBU</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1001,7 +989,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>NBU gross international reserves (preliminary)</t>
+          <t>NBU gross international reserves</t>
         </is>
       </c>
     </row>
@@ -1011,16 +999,34 @@
           <t>net_reserves_usd_bn</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n"/>
+      <c r="B17" s="2" t="n">
+        <v>38.6</v>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>USD bn</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>IMF reserve template</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>net of predetermined and contingent one-year drains</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1043,7 +1049,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>National Bank of Ukraine</t>
+          <t>NBU</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1111,7 +1117,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>225.337</v>
+        <v>225.3</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1133,11 +1139,7 @@
           <t>08-Oct-26</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1293,11 +1295,8 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Extended Fund Facility (EFF), 4-year</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>15.6</v>
+          <t>4-year EFF (first review completed 20-Jul-26, SDR 503M, about $690M disbursed)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1346,8 +1345,14 @@
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" t="inlineStr"/>
+      <c r="C2" s="2" t="n">
+        <v>225.3</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1356,8 +1361,14 @@
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" t="inlineStr"/>
+      <c r="C3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1376,8 +1387,14 @@
         </is>
       </c>
       <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" t="inlineStr"/>
+      <c r="C5" s="2" t="n">
+        <v>-18.9</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1386,8 +1403,14 @@
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" t="inlineStr"/>
+      <c r="C6" s="2" t="n">
+        <v>-18.4</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>IMF WEO, 08-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1411,7 +1434,7 @@
       <c r="C8" s="2" t="n"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ministry of Finance of Ukraine, 31-Dec-25</t>
+          <t>Ministry of Finance of Ukraine (state debt), 31-Dec-25</t>
         </is>
       </c>
     </row>

</xml_diff>